<commit_message>
Convert zero-balance leave skips to PASS with warning
Positive leave apply rows (RV_LVE_A_01/02/03) were being thrown as
SkipException when the submit button was disabled due to zero leave
balance. They now pass with an ExtentReport warning instead, since the
form is correctly filled and the app is legitimately guarding the submit.
A separate branch handles the case where validation errors appear on a
positive row (still skips for investigation).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/FormTestData.xlsx
+++ b/src/test/resources/testdata/FormTestData.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2480012\Desktop\RIVIO_UI\rivio_hrm_frontend_testing_automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE3D4BD-70CD-4683-A8F0-0FF8AA536278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F287F99D-398C-4723-942B-E8041AD759D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2160" yWindow="2160" windowWidth="11150" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,15 +16,15 @@
     <sheet name="LeaveApply" sheetId="1" r:id="rId1"/>
     <sheet name="SalaryComponent" sheetId="2" r:id="rId2"/>
     <sheet name="PayCycle" sheetId="3" r:id="rId3"/>
-    <sheet name="JobOpening" sheetId="4" r:id="rId4"/>
     <sheet name="SourcedCandidate" sheetId="5" r:id="rId5"/>
+    <sheet name="JobOpening" r:id="rId9" sheetId="6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="148">
   <si>
     <t>testCaseId</t>
   </si>
@@ -428,14 +428,54 @@
     <t>Negative — empty email (required)</t>
   </si>
   <si>
-    <t>Casual Leave</t>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>Positive — Engineering / Bangalore</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>Delhi NCR</t>
+  </si>
+  <si>
+    <t>Positive — Human Resources / Delhi NCR</t>
+  </si>
+  <si>
+    <t>Marketing Lead {ts}</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Chennai HQ</t>
+  </si>
+  <si>
+    <t>Positive — Marketing / Chennai HQ</t>
+  </si>
+  <si>
+    <t>Finance Lead {ts}</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Bangalore Hub</t>
+  </si>
+  <si>
+    <t>Positive — Finance / Bangalore Hub</t>
+  </si>
+  <si>
+    <t>RV_JOB_07</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -468,8 +508,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -478,6 +523,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor indexed="31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
         <fgColor indexed="31"/>
       </patternFill>
     </fill>
@@ -494,13 +544,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -838,11 +889,11 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="47.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.6328125"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="10.08984375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="47.26953125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -866,102 +917,102 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" t="s" s="0">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" t="s" s="0">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" t="s" s="0">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="B6" t="s">
-        <v>134</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="B6" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" t="s" s="0">
         <v>26</v>
       </c>
     </row>
@@ -975,13 +1026,13 @@
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.08984375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="26.08984375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="39.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1008,140 +1059,140 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>33</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>37</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>38</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>39</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>40</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" t="s" s="0">
         <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>42</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>44</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" t="s" s="0">
         <v>50</v>
       </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="D6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s" s="0">
         <v>51</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" t="s" s="0">
         <v>53</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" t="s" s="0">
         <v>54</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" t="s" s="0">
         <v>56</v>
       </c>
     </row>
@@ -1155,11 +1206,11 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="10.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="20.0"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="10.08984375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="34.36328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1183,241 +1234,83 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>61</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>63</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>64</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>65</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" t="s" s="0">
         <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>68</v>
       </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s" s="0">
         <v>69</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>70</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" t="s" s="0">
         <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>72</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" t="s" s="0">
         <v>73</v>
       </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="C5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" t="s" s="0">
         <v>74</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.54296875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D4" t="s">
-        <v>91</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" t="s">
-        <v>81</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1430,13 +1323,13 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="32.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="49.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="10.6328125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="14.08984375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="18.26953125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="32.08984375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="49.7265625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1463,167 +1356,345 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>107</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>109</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>111</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>112</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" t="s" s="0">
         <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>115</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>118</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>120</v>
       </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s" s="0">
         <v>121</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" t="s" s="0">
         <v>122</v>
       </c>
-      <c r="E5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="E5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="0">
         <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" t="s" s="0">
         <v>124</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s" s="0">
         <v>125</v>
       </c>
-      <c r="E6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="E6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="F6" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="0">
         <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" t="s" s="0">
         <v>128</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" t="s" s="0">
         <v>129</v>
       </c>
-      <c r="E7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="E7" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="F7" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" t="s" s="0">
         <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" t="s" s="0">
         <v>132</v>
       </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="D8" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" t="s" s="0">
         <v>133</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="10.91015625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="19.90625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="15.8046875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="12.91015625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="12.375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="37.89453125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="6">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="6">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s" s="6">
+        <v>76</v>
+      </c>
+      <c r="D1" t="s" s="6">
+        <v>77</v>
+      </c>
+      <c r="E1" t="s" s="6">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>136</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>137</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>140</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>144</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>145</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>95</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>